<commit_message>
Enhance course name normalization and update related documents
- Added regex to handle Swedish elliptic-compound hyphens in course names for better normalization in both `checks_nedlagda.py` and `scrape_hda_utbildningsplaner.py`.
- Updated the download links and row counts in markdown files for "Nedlagda kursreferenser" and "Stavfel och språkbruk" across multiple directories.
- Modified various Excel files related to grading reports, grading scales, Bloom taxonomy, examination forms, phrasing consistency, and knowledge requirements in all university departments (IIT, IHV, IKS, ISLL).
</commit_message>
<xml_diff>
--- a/vault-dalarna-university/01 IIT/Analys/Nedlagda kursreferenser.xlsx
+++ b/vault-dalarna-university/01 IIT/Analys/Nedlagda kursreferenser.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Nedlagda kursreferenser" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Nedlagda kursreferenser'!$A$1:$E$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Nedlagda kursreferenser'!$A$1:$E$16</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -472,7 +472,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>DITMG</t>
+          <t>TATPG</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -487,19 +487,19 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>`System- och verksamhetsutveckling` → `GIK2JW` (nedlagd 2025-12-08) — plain-text-referens; rad: - System- och verksamhetsutveckling, 7,5hp</t>
+          <t>`Produktutveckling` → `MT2016` (nedlagd 2021-11-30) — plain-text-referens; rad: - Produktutveckling, 7,5 hp</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=DITMG</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TATPG</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>DSVPG</t>
+          <t>TPOKG</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -514,19 +514,19 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>`System- och verksamhetsutveckling` → `GIK2JW` (nedlagd 2025-12-08) — plain-text-referens; rad: - System- och verksamhetsutveckling, 7,5 hp</t>
+          <t>`Industriell Ekonomi med kalkylering` → `IE1062` (nedlagd 2024-11-06) — plain-text-referens; rad: - Industriell Ekonomi med kalkylering, 7,5hp</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=DSVPG</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TPOKG</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>KGDWG</t>
+          <t>TPOKG</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -541,19 +541,19 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>`System- och verksamhetsutveckling` → `GIK2JW` (nedlagd 2025-12-08) — plain-text-referens; rad: - System- och verksamhetsutveckling, 7,5 hp</t>
+          <t>`Introduktion till mekanik och hållfasthetslära` → `MT1067` (nedlagd 2025-12-08) — plain-text-referens; rad: - Introduktion till mekanik och hållfasthetslära, 7,5hp</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=KGDWG</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TPOKG</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>TATPG</t>
+          <t>TPOKG</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -568,12 +568,12 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>`Produktutveckling` → `MT2016` (nedlagd 2021-11-30) — plain-text-referens; rad: - Produktutveckling, 7,5 hp</t>
+          <t>`3D CAD Grundläggande` → `MT1051` (nedlagd 2025-08-21) — plain-text-referens; rad: - 3D CAD Grundläggande, 7,5hp</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TATPG</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TPOKG</t>
         </is>
       </c>
     </row>
@@ -595,7 +595,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>`Industriell Ekonomi med kalkylering` → `IE1062` (nedlagd 2024-11-06) — plain-text-referens; rad: - Industriell Ekonomi med kalkylering, 7,5hp</t>
+          <t>`Statistik för ingenjörer` → `ST1028` (nedlagd 2024-11-06) — plain-text-referens; rad: - Statistik för ingenjörer, 7,5hp</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -622,7 +622,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>`Introduktion till mekanik och hållfasthetslära` → `MT1067` (nedlagd 2025-12-08) — plain-text-referens; rad: - Introduktion till mekanik och hållfasthetslära, 7,5hp</t>
+          <t>`Tillverkningsteknik` → `MT1070` (nedlagd 2025-12-08) — plain-text-referens; rad: - Tillverkningsteknik, 7,5hp</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -649,7 +649,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>`3D CAD Grundläggande` → `MT1051` (nedlagd 2025-08-21) — plain-text-referens; rad: - 3D CAD Grundläggande, 7,5hp</t>
+          <t>`Grundläggande materiallära` → `GMP2LL` (nedlagd 2025-09-30) — plain-text-referens; rad: - Grundläggande materiallära, 7,5hp</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -676,7 +676,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>`Statistik för ingenjörer` → `ST1028` (nedlagd 2024-11-06) — plain-text-referens; rad: - Statistik för ingenjörer, 7,5hp</t>
+          <t>`CAD/CAM` → `MT1072` (nedlagd 2025-12-08) — plain-text-referens; rad: - CAD/CAM, 7,5hp</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -703,7 +703,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>`Tillverkningsteknik` → `MT1070` (nedlagd 2025-12-08) — plain-text-referens; rad: - Tillverkningsteknik, 7,5hp</t>
+          <t>`Hydraulik och Pneumatik` → `MT1073` (nedlagd 2025-12-08) — plain-text-referens; rad: - Hydraulik och Pneumatik, 7,5hp</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -730,7 +730,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>`Grundläggande materiallära` → `GMP2LL` (nedlagd 2025-09-30) — plain-text-referens; rad: - Grundläggande materiallära, 7,5hp</t>
+          <t>`Grundläggande ellära för maskinteknik` → `ET1022` (nedlagd 2024-11-06) — plain-text-referens; rad: - Grundläggande ellära för maskinteknik, 3,5hp</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -757,7 +757,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>`CAD/CAM` → `MT1072` (nedlagd 2025-12-08) — plain-text-referens; rad: - CAD/CAM, 7,5hp</t>
+          <t>`Materialval` → `MP2039` (nedlagd 2025-09-30) — plain-text-referens; rad: - Materialval, 4hp</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -784,7 +784,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>`Hydraulik och Pneumatik` → `MT1073` (nedlagd 2025-12-08) — plain-text-referens; rad: - Hydraulik och Pneumatik, 7,5hp</t>
+          <t>`Introduktion till hållbar utveckling inom maskinteknik` → `GMT2CU` (nedlagd 2025-12-08) — plain-text-referens; rad: - Introduktion till hållbar utveckling inom maskinteknik, 7,5hp</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -811,7 +811,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>`Grundläggande ellära för maskinteknik` → `ET1022` (nedlagd 2024-11-06) — plain-text-referens; rad: - Grundläggande ellära för maskinteknik, 3,5hp</t>
+          <t>`Konstruktionsprojekt` → `GMT224` (nedlagd 2025-12-08) — plain-text-referens; rad: - Konstruktionsprojekt, 7,5hp</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -838,7 +838,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>`Materialval` → `MP2039` (nedlagd 2025-09-30) — plain-text-referens; rad: - Materialval, 4hp</t>
+          <t>`Kvalitetsteknik` → `GMT2CV` (nedlagd 2025-12-08) — plain-text-referens; rad: - Kvalitetsteknik, 7,5hp</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -865,7 +865,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>`Introduktion till hållbar utveckling inom maskinteknik` → `GMT2CU` (nedlagd 2025-12-08) — plain-text-referens; rad: - Introduktion till hållbar utveckling inom maskinteknik, 7,5hp</t>
+          <t>`Industriell produktion` → `GMT259` (nedlagd 2025-12-08) — plain-text-referens; rad: - Industriell produktion, 7,5hp</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -874,89 +874,8 @@
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>TPOKG</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Utbildningsplan</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Programmet listar nedlagd kurs</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>`Konstruktionsprojekt` → `GMT224` (nedlagd 2025-12-08) — plain-text-referens; rad: - Konstruktionsprojekt, 7,5hp</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TPOKG</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>TPOKG</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Utbildningsplan</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Programmet listar nedlagd kurs</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>`Kvalitetsteknik` → `GMT2CV` (nedlagd 2025-12-08) — plain-text-referens; rad: - Kvalitetsteknik, 7,5hp</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TPOKG</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>TPOKG</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Utbildningsplan</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Programmet listar nedlagd kurs</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>`Industriell produktion` → `GMT259` (nedlagd 2025-12-08) — plain-text-referens; rad: - Industriell produktion, 7,5hp</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TPOKG</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:E19"/>
+  <autoFilter ref="A1:E16"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId2"/>
@@ -988,12 +907,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId28"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A16" r:id="rId29"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A17" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A18" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A19" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId36"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>